<commit_message>
Add lab ideas, textbook comparison, and schedule updates
Sketch out labs 1-5 by topic, compare the Chapra & Canale and Chapra
textbook outlines, and update the draft schedule.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="69">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -58,7 +58,7 @@
     <t xml:space="preserve">W</t>
   </si>
   <si>
-    <t xml:space="preserve">Algorithms and Estimating Time Complexity</t>
+    <t xml:space="preserve">Algorithms and Time Complexity</t>
   </si>
   <si>
     <t xml:space="preserve">Lab 0: Implementing Algorithms</t>
@@ -100,21 +100,21 @@
     <t xml:space="preserve">Nonlinear Algebraic Equations</t>
   </si>
   <si>
+    <t xml:space="preserve">Lab 2: Interactive Algorithm Lab ???</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed Point Iteration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Newton’s Method</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lab 2: Solving Nonlinear Systems</t>
   </si>
   <si>
-    <t xml:space="preserve">Fixed Point Iteration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Newton’s Method</t>
-  </si>
-  <si>
     <t xml:space="preserve">Exam 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Code Interview 1</t>
-  </si>
-  <si>
     <t xml:space="preserve">Euler’s Method</t>
   </si>
   <si>
@@ -124,15 +124,15 @@
     <t xml:space="preserve">Also, exact solutions to linear </t>
   </si>
   <si>
+    <t xml:space="preserve">Lab 3: Simulating ODEs</t>
+  </si>
+  <si>
     <t xml:space="preserve">Runge-Kutta Methods</t>
   </si>
   <si>
     <t xml:space="preserve">Including adaptive Runge-Kutta</t>
   </si>
   <si>
-    <t xml:space="preserve">Lab 3: Simulating ODEs</t>
-  </si>
-  <si>
     <t xml:space="preserve">Stiff equations and Implicit integration</t>
   </si>
   <si>
@@ -145,48 +145,48 @@
     <t xml:space="preserve">Optimization</t>
   </si>
   <si>
+    <t xml:space="preserve">Gradient Descent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Line Search, Momentum, ADAM</t>
+  </si>
+  <si>
     <t xml:space="preserve">Should be Review, Necessary and sufficient conditions for optimality</t>
   </si>
   <si>
-    <t xml:space="preserve">Gradient Descent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Line Search, Momentum, ADAM</t>
-  </si>
-  <si>
     <t xml:space="preserve">Lab 4: Optimization</t>
   </si>
   <si>
+    <t xml:space="preserve">Exam 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Constrained Optimization: Lagrange Multipliers</t>
+  </si>
+  <si>
     <t xml:space="preserve">Maybe also touch on Quasi-Newton/Conjugate Gradient</t>
   </si>
   <si>
-    <t xml:space="preserve">Constrained Optimization: Lagrange Multipliers</t>
+    <t xml:space="preserve">Interior point methods</t>
   </si>
   <si>
     <t xml:space="preserve">Neither book talks about constraints</t>
   </si>
   <si>
-    <t xml:space="preserve">Interior point methods</t>
+    <t xml:space="preserve">Regression problems and least-squares</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regression and Learning</t>
   </si>
   <si>
     <t xml:space="preserve">Could alternatively do Augmented Lagrangian, but I think interior point has the best </t>
   </si>
   <si>
-    <t xml:space="preserve">Exam 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Regression problems and least-squares</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Regression and Learning</t>
+    <t xml:space="preserve">Least-squares with nonlinear basis functions</t>
   </si>
   <si>
     <t xml:space="preserve">R-squared value</t>
   </si>
   <si>
-    <t xml:space="preserve">Least-squares with nonlinear basis functions</t>
-  </si>
-  <si>
     <t xml:space="preserve">Lab 5: Regression</t>
   </si>
   <si>
@@ -197,6 +197,9 @@
   </si>
   <si>
     <t xml:space="preserve">Gradients of Neural Network Parameters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exam 3</t>
   </si>
   <si>
     <t xml:space="preserve">THANKSGIVING BREAK</t>
@@ -289,7 +292,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -310,8 +313,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFB66C"/>
+        <bgColor rgb="FFFFAB91"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFAB91"/>
-        <bgColor rgb="FFFFCC99"/>
+        <bgColor rgb="FFFFB66C"/>
       </patternFill>
     </fill>
     <fill>
@@ -361,7 +370,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -402,18 +411,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -422,11 +423,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -493,7 +506,7 @@
       <rgbColor rgb="FF90CAF9"/>
       <rgbColor rgb="FFFFAB91"/>
       <rgbColor rgb="FFCE93D8"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFFFB66C"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -523,34 +536,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -696,7 +709,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F49"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="6"/>
@@ -721,7 +734,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="n">
         <v>46255</v>
       </c>
@@ -736,7 +749,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="n">
         <v>46258</v>
       </c>
@@ -751,7 +764,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="n">
         <v>46260</v>
       </c>
@@ -764,7 +777,7 @@
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
     </row>
-    <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="n">
         <v>46262</v>
       </c>
@@ -777,7 +790,7 @@
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
     </row>
-    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="n">
         <v>46265</v>
       </c>
@@ -795,7 +808,7 @@
       </c>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="n">
         <v>46267</v>
       </c>
@@ -808,7 +821,7 @@
       <c r="D7" s="7"/>
       <c r="E7" s="4"/>
     </row>
-    <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="n">
         <v>46269</v>
       </c>
@@ -821,7 +834,7 @@
       <c r="D8" s="7"/>
       <c r="E8" s="4"/>
     </row>
-    <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="n">
         <v>46272</v>
       </c>
@@ -836,7 +849,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="n">
         <v>46274</v>
       </c>
@@ -847,9 +860,8 @@
         <v>21</v>
       </c>
       <c r="D10" s="7"/>
-      <c r="E10" s="0"/>
-    </row>
-    <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="n">
         <v>46276</v>
       </c>
@@ -862,14 +874,14 @@
       <c r="D11" s="7"/>
       <c r="E11" s="4"/>
     </row>
-    <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="n">
         <v>46279</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="1" t="s">
         <v>22</v>
       </c>
       <c r="D12" s="7"/>
@@ -877,7 +889,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="n">
         <v>46281</v>
       </c>
@@ -892,7 +904,7 @@
       </c>
       <c r="E13" s="4"/>
     </row>
-    <row r="14" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="n">
         <v>46283</v>
       </c>
@@ -905,7 +917,7 @@
       <c r="D14" s="9"/>
       <c r="E14" s="4"/>
     </row>
-    <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="n">
         <v>46286</v>
       </c>
@@ -918,7 +930,7 @@
       <c r="D15" s="9"/>
       <c r="E15" s="4"/>
     </row>
-    <row r="16" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="n">
         <v>46288</v>
       </c>
@@ -931,7 +943,7 @@
       <c r="D16" s="9"/>
       <c r="E16" s="4"/>
     </row>
-    <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="n">
         <v>46290</v>
       </c>
@@ -939,36 +951,42 @@
         <v>5</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D17" s="9"/>
       <c r="E17" s="4"/>
     </row>
-    <row r="18" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="n">
         <v>46293</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C18" s="4" t="s">
-        <v>29</v>
+      <c r="C18" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
     </row>
-    <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="n">
         <v>46295</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-    </row>
-    <row r="20" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C19" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="n">
         <v>46297</v>
       </c>
@@ -976,12 +994,12 @@
         <v>5</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="D20" s="4"/>
+        <v>34</v>
+      </c>
+      <c r="D20" s="12"/>
       <c r="E20" s="4"/>
     </row>
-    <row r="21" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="n">
         <v>46300</v>
       </c>
@@ -989,31 +1007,27 @@
         <v>8</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D21" s="10" t="s">
-        <v>32</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="D21" s="12"/>
       <c r="E21" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="n">
         <v>46302</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C22" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="D22" s="11"/>
-      <c r="E22" s="4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C22" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D22" s="12"/>
+      <c r="E22" s="0"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="n">
         <v>46304</v>
       </c>
@@ -1021,38 +1035,40 @@
         <v>5</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D23" s="11"/>
+        <v>34</v>
+      </c>
+      <c r="D23" s="12"/>
       <c r="E23" s="4"/>
     </row>
-    <row r="24" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="n">
         <v>46307</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C24" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D24" s="11"/>
+      <c r="C24" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D24" s="12"/>
       <c r="E24" s="4"/>
     </row>
-    <row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="n">
         <v>46309</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C25" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="D25" s="11"/>
+      <c r="C25" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>40</v>
+      </c>
       <c r="E25" s="4"/>
     </row>
-    <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="n">
         <v>46311</v>
       </c>
@@ -1060,40 +1076,40 @@
         <v>5</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D26" s="11"/>
+        <v>34</v>
+      </c>
+      <c r="D26" s="13"/>
       <c r="E26" s="4"/>
     </row>
-    <row r="27" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="n">
         <v>46314</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C27" s="4"/>
-      <c r="D27" s="12"/>
+      <c r="C27" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D27" s="14"/>
       <c r="E27" s="4"/>
     </row>
-    <row r="28" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="n">
         <v>46316</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C28" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D28" s="13" t="s">
-        <v>40</v>
-      </c>
+      <c r="C28" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D28" s="14"/>
       <c r="E28" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="n">
         <v>46318</v>
       </c>
@@ -1101,25 +1117,25 @@
         <v>5</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="D29" s="14"/>
       <c r="E29" s="4"/>
     </row>
-    <row r="30" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="n">
         <v>46321</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C30" s="4" t="s">
-        <v>42</v>
+      <c r="C30" s="15" t="s">
+        <v>45</v>
       </c>
       <c r="D30" s="14"/>
       <c r="E30" s="4"/>
     </row>
-    <row r="31" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="n">
         <v>46323</v>
       </c>
@@ -1127,11 +1143,11 @@
         <v>11</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="D31" s="14"/>
     </row>
-    <row r="32" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="n">
         <v>46325</v>
       </c>
@@ -1143,7 +1159,7 @@
       </c>
       <c r="D32" s="14"/>
     </row>
-    <row r="33" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="n">
         <v>46328</v>
       </c>
@@ -1151,14 +1167,14 @@
         <v>8</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="D33" s="14"/>
       <c r="E33" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="n">
         <v>46330</v>
       </c>
@@ -1166,14 +1182,14 @@
         <v>11</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D34" s="14"/>
       <c r="E34" s="4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="n">
         <v>46332</v>
       </c>
@@ -1183,9 +1199,9 @@
       <c r="C35" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="D35" s="14"/>
-    </row>
-    <row r="36" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D35" s="0"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="n">
         <v>46335</v>
       </c>
@@ -1193,25 +1209,31 @@
         <v>8</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="D36" s="14"/>
+        <v>50</v>
+      </c>
+      <c r="D36" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="E36" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="n">
         <v>46337</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C37" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C37" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D37" s="17"/>
+      <c r="E37" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="n">
         <v>46339</v>
       </c>
@@ -1219,11 +1241,12 @@
         <v>5</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>44</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="D38" s="17"/>
       <c r="E38" s="4"/>
     </row>
-    <row r="39" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="n">
         <v>46342</v>
       </c>
@@ -1231,16 +1254,14 @@
         <v>8</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="D39" s="15" t="s">
-        <v>52</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="D39" s="17"/>
       <c r="E39" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="n">
         <v>46344</v>
       </c>
@@ -1248,12 +1269,12 @@
         <v>11</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="D40" s="16"/>
+        <v>58</v>
+      </c>
+      <c r="D40" s="17"/>
       <c r="E40" s="4"/>
     </row>
-    <row r="41" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="n">
         <v>46346</v>
       </c>
@@ -1263,38 +1284,34 @@
       <c r="C41" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="D41" s="16"/>
+      <c r="D41" s="0"/>
       <c r="E41" s="4"/>
     </row>
-    <row r="42" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="n">
         <v>46349</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C42" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="D42" s="16"/>
-      <c r="E42" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C42" s="0"/>
+      <c r="D42" s="0"/>
+      <c r="E42" s="0"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="n">
         <v>46351</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C43" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="D43" s="16"/>
+      <c r="C43" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D43" s="0"/>
       <c r="E43" s="4"/>
     </row>
-    <row r="44" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="n">
         <v>46353</v>
       </c>
@@ -1302,12 +1319,12 @@
         <v>5</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="D44" s="16"/>
+        <v>60</v>
+      </c>
+      <c r="D44" s="17"/>
       <c r="E44" s="4"/>
     </row>
-    <row r="45" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="n">
         <v>46356</v>
       </c>
@@ -1315,12 +1332,12 @@
         <v>8</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D45" s="16"/>
+        <v>61</v>
+      </c>
+      <c r="D45" s="17"/>
       <c r="E45" s="4"/>
     </row>
-    <row r="46" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="n">
         <v>46358</v>
       </c>
@@ -1328,51 +1345,46 @@
         <v>11</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D46" s="16"/>
+        <v>62</v>
+      </c>
+      <c r="D46" s="17"/>
       <c r="E46" s="4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="n">
         <v>46360</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="D47" s="16"/>
+        <v>65</v>
+      </c>
+      <c r="D47" s="17"/>
       <c r="E47" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="17" t="n">
+      <c r="A49" s="18" t="n">
         <v>46365</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:B47 C23 E22 C38:C47 C25:C27 C29:C36 C13:C21 C2:C11">
+  <conditionalFormatting sqref="A2:B47 C23:C24 C2:C11 C26:C29 C13:C21 E21 C31:C41 C44:C47">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>$B2="F"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C22">
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>$B22="F"</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>